<commit_message>
fix: force vercel redeploy
</commit_message>
<xml_diff>
--- a/autohogar/5_EXCELS_SISTEMA_LOCAL/BASE_MAESTRA_AUTOHOGAR_NUBE.xlsx
+++ b/autohogar/5_EXCELS_SISTEMA_LOCAL/BASE_MAESTRA_AUTOHOGAR_NUBE.xlsx
@@ -400,26 +400,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:R196"/>
-  <cols>
-    <col min="1" max="1" width="35.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="35.83203125" customWidth="1"/>
-    <col min="4" max="4" width="25.83203125" customWidth="1"/>
-    <col min="5" max="5" width="30.83203125" customWidth="1"/>
-    <col min="6" max="6" width="20.83203125" customWidth="1"/>
-    <col min="7" max="7" width="15.83203125" customWidth="1"/>
-    <col min="8" max="8" width="15.83203125" customWidth="1"/>
-    <col min="9" max="9" width="35.83203125" customWidth="1"/>
-    <col min="10" max="10" width="25.83203125" customWidth="1"/>
-    <col min="11" max="11" width="20.83203125" customWidth="1"/>
-    <col min="12" max="12" width="22.83203125" customWidth="1"/>
-    <col min="13" max="13" width="20.83203125" customWidth="1"/>
-    <col min="14" max="14" width="20.83203125" customWidth="1"/>
-    <col min="15" max="15" width="25.83203125" customWidth="1"/>
-    <col min="16" max="16" width="25.83203125" customWidth="1"/>
-    <col min="17" max="17" width="40.83203125" customWidth="1"/>
-    <col min="18" max="18" width="40.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4720,8 +4700,8 @@
       <c r="N77" t="str">
         <v>ELECTRONICO</v>
       </c>
-      <c r="O77" t="str">
-        <v/>
+      <c r="O77">
+        <v>-118000</v>
       </c>
       <c r="P77" t="str">
         <v/>
@@ -4730,7 +4710,7 @@
         <v/>
       </c>
       <c r="R77" t="str">
-        <v/>
+        <v>BAJA Y DEVOLUCION</v>
       </c>
     </row>
     <row r="78">
@@ -8360,8 +8340,8 @@
       <c r="N142" t="str">
         <v>ELECTRONICO</v>
       </c>
-      <c r="O142" t="str">
-        <v/>
+      <c r="O142">
+        <v>60000</v>
       </c>
       <c r="P142" t="str">
         <v/>
@@ -8370,7 +8350,7 @@
         <v/>
       </c>
       <c r="R142" t="str">
-        <v/>
+        <v>BAJA POR FALTADE PAGO Y COMUNICACIÓN</v>
       </c>
     </row>
     <row r="143">
@@ -8920,8 +8900,8 @@
       <c r="N152" t="str">
         <v>ELECTRONICO</v>
       </c>
-      <c r="O152" t="str">
-        <v/>
+      <c r="O152">
+        <v>15000</v>
       </c>
       <c r="P152" t="str">
         <v/>
@@ -9424,8 +9404,8 @@
       <c r="N161" t="str">
         <v>ELECTRONICO</v>
       </c>
-      <c r="O161" t="str">
-        <v/>
+      <c r="O161">
+        <v>60000</v>
       </c>
       <c r="P161" t="str">
         <v/>
@@ -9434,7 +9414,7 @@
         <v/>
       </c>
       <c r="R161" t="str">
-        <v/>
+        <v>MERCADO PAGO</v>
       </c>
     </row>
     <row r="162">
@@ -10264,8 +10244,8 @@
       <c r="N176" t="str">
         <v>ELECTRONICO</v>
       </c>
-      <c r="O176" t="str">
-        <v/>
+      <c r="O176">
+        <v>-13</v>
       </c>
       <c r="P176" t="str">
         <v/>
@@ -10600,8 +10580,8 @@
       <c r="N182" t="str">
         <v>ELECTRONICO</v>
       </c>
-      <c r="O182" t="str">
-        <v/>
+      <c r="O182">
+        <v>-60000</v>
       </c>
       <c r="P182" t="str">
         <v/>
@@ -11338,7 +11318,7 @@
         <v/>
       </c>
       <c r="R195" t="str">
-        <v/>
+        <v>BAJA INFORMA EDUARDO</v>
       </c>
     </row>
     <row r="196">
@@ -11407,16 +11387,6 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H1"/>
-  <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="35.83203125" customWidth="1"/>
-    <col min="4" max="4" width="25.83203125" customWidth="1"/>
-    <col min="5" max="5" width="20.83203125" customWidth="1"/>
-    <col min="6" max="6" width="20.83203125" customWidth="1"/>
-    <col min="7" max="7" width="40.83203125" customWidth="1"/>
-    <col min="8" max="8" width="35.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -11454,16 +11424,6 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H2"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="35.83203125" customWidth="1"/>
-    <col min="5" max="5" width="35.83203125" customWidth="1"/>
-    <col min="6" max="6" width="30.83203125" customWidth="1"/>
-    <col min="7" max="7" width="35.83203125" customWidth="1"/>
-    <col min="8" max="8" width="40.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">

</xml_diff>